<commit_message>
Full name of resource in average table
</commit_message>
<xml_diff>
--- a/source/BossDrops.xlsx
+++ b/source/BossDrops.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1337c\OneDrive\Skrivbord\Projects\Nebula calc\source\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ulrika\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B5841D9C-4607-48A8-A9FC-D3B88AA103D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B49A6A-A7C6-4B1E-BB96-4241FE87D393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" xr2:uid="{D55BD798-421B-4B04-AA33-88A80DD2AC5C}"/>
+    <workbookView xWindow="28680" yWindow="-2025" windowWidth="29040" windowHeight="17520" xr2:uid="{D55BD798-421B-4B04-AA33-88A80DD2AC5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Lords" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="20">
   <si>
     <t>Nubhe</t>
   </si>
@@ -85,12 +85,27 @@
   <si>
     <t>Attempts</t>
   </si>
+  <si>
+    <t>Primary Shard</t>
+  </si>
+  <si>
+    <t>Intermediate Shard</t>
+  </si>
+  <si>
+    <t>Advanced Shard</t>
+  </si>
+  <si>
+    <t>Primary Essence</t>
+  </si>
+  <si>
+    <t>Intermediate Essence</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -107,6 +122,30 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="7"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -138,13 +177,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -163,7 +206,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -480,12 +523,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D19CB3BD-8C90-46B6-8962-159A436E4641}">
   <dimension ref="A1:SG64"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="501" width="10.6640625" customWidth="1"/>
+    <col min="1" max="501" width="10.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:501" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1990,7 +2033,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="2" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2352,7 +2395,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2714,7 +2757,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -3076,7 +3119,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -3330,7 +3373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -3458,12 +3501,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:501" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -4968,7 +5011,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="9" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -5456,7 +5499,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -5944,7 +5987,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -6432,7 +6475,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -6764,7 +6807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -6982,12 +7025,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:501" ht="15" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
@@ -8492,7 +8535,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="16" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -9097,7 +9140,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -9702,7 +9745,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>3</v>
       </c>
@@ -10307,7 +10350,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -10777,7 +10820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -11031,12 +11074,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:501" ht="15" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
@@ -12541,7 +12584,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="23" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>1</v>
       </c>
@@ -13155,7 +13198,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>2</v>
       </c>
@@ -13769,7 +13812,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>3</v>
       </c>
@@ -14383,7 +14426,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -14853,7 +14896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>5</v>
       </c>
@@ -15113,12 +15156,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:501" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>10</v>
       </c>
@@ -16623,7 +16666,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="30" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>1</v>
       </c>
@@ -17384,7 +17427,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>2</v>
       </c>
@@ -18145,7 +18188,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>3</v>
       </c>
@@ -18906,7 +18949,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -19496,7 +19539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>5</v>
       </c>
@@ -19834,12 +19877,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:501" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>11</v>
       </c>
@@ -21344,7 +21387,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="37" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>1</v>
       </c>
@@ -22702,7 +22745,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="38" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>2</v>
       </c>
@@ -24060,7 +24103,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>3</v>
       </c>
@@ -25418,7 +25461,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="40" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -26395,7 +26438,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>5</v>
       </c>
@@ -26919,12 +26962,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:501" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>12</v>
       </c>
@@ -28429,7 +28472,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="44" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>1</v>
       </c>
@@ -29793,7 +29836,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="45" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>2</v>
       </c>
@@ -31157,7 +31200,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="46" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>3</v>
       </c>
@@ -32521,7 +32564,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -33561,7 +33604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:501" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:501" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>5</v>
       </c>
@@ -34082,12 +34125,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>13</v>
       </c>
@@ -34113,7 +34156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>14</v>
       </c>
@@ -34139,9 +34182,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>1</v>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="B53">
         <f>SUM(B44:QL44)</f>
@@ -34172,7 +34215,7 @@
         <v>3473</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>13</v>
       </c>
@@ -34205,9 +34248,9 @@
         <v>29.184873949579831</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>2</v>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="B55">
         <f>SUM(B45:QL45)</f>
@@ -34238,7 +34281,7 @@
         <v>2969</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>13</v>
       </c>
@@ -34271,9 +34314,9 @@
         <v>24.949579831932773</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>3</v>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="B57">
         <f>SUM(B46:QL46)</f>
@@ -34304,7 +34347,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>13</v>
       </c>
@@ -34337,9 +34380,9 @@
         <v>3.9327731092436973</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>4</v>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="B59">
         <f>SUM(B47:QL47)</f>
@@ -34370,7 +34413,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>13</v>
       </c>
@@ -34403,9 +34446,9 @@
         <v>0.96638655462184875</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>5</v>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" s="6" t="s">
+        <v>19</v>
       </c>
       <c r="B61">
         <f>SUM(B48:QL48)</f>
@@ -34436,7 +34479,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" ht="15" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>13</v>
       </c>
@@ -34469,7 +34512,7 @@
         <v>0.34453781512605042</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E64" s="3"/>
     </row>
   </sheetData>

</xml_diff>